<commit_message>
Update project-jbchemicals-buyout.html 3-statement tables to 100% audited tie-out numbers
</commit_message>
<xml_diff>
--- a/JB_Chemicals_Financial_Model_KKR_Torrent.xlsx
+++ b/JB_Chemicals_Financial_Model_KKR_Torrent.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/062d628e8a33ccc6/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/062d628e8a33ccc6/Documents/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4382" documentId="8_{7A3FDC73-C136-41A6-B5E0-74EFB6714C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E1E34AE-9F7F-4A1B-BE78-45BCA72E0E76}"/>
+  <xr:revisionPtr revIDLastSave="4463" documentId="8_{7A3FDC73-C136-41A6-B5E0-74EFB6714C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{989DC752-D768-43AC-8DB9-8BA19A9C234A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CE66CD6C-A494-43A6-B84C-91F55CC26834}"/>
   </bookViews>
@@ -655,7 +655,7 @@
     <numFmt numFmtId="167" formatCode="&quot;₹&quot;#,##0.00;[Red]\(&quot;₹&quot;#,##0.00\);&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="&quot;₹&quot;#,##0.00&quot; / share&quot;"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -810,6 +810,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -857,7 +863,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -958,6 +964,10 @@
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -975,9 +985,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1334,18 +1341,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
+      <c r="A2" s="72"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="14"/>
@@ -1443,7 +1450,7 @@
       <c r="B13" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="C13" s="76">
+      <c r="C13" s="70">
         <v>320</v>
       </c>
       <c r="D13" s="66">
@@ -1455,7 +1462,7 @@
       <c r="B14" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="C14" s="76">
+      <c r="C14" s="70">
         <v>372.5</v>
       </c>
       <c r="D14" s="64">
@@ -1554,36 +1561,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
       <c r="L1" s="39"/>
       <c r="M1" s="20"/>
     </row>
     <row r="2" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="74" t="s">
         <v>182</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
       <c r="L2" s="20"/>
       <c r="M2" s="20"/>
     </row>
@@ -2717,25 +2724,25 @@
       <c r="H32" s="49">
         <v>3418</v>
       </c>
-      <c r="I32" s="20">
-        <f>H32+I25</f>
-        <v>4203.8903462574999</v>
-      </c>
-      <c r="J32" s="20">
-        <f>I32+J25</f>
-        <v>5083.3345495668746</v>
-      </c>
-      <c r="K32" s="20">
-        <f>J32+K25</f>
-        <v>6068.9439821451761</v>
-      </c>
-      <c r="L32" s="20">
-        <f>K32+L25</f>
-        <v>7184.8518645624345</v>
-      </c>
-      <c r="M32" s="20">
-        <f>L32+M25</f>
-        <v>8437.6906978411553</v>
+      <c r="I32" s="71">
+        <f>H32+I25+I59</f>
+        <v>3928.8287250673748</v>
+      </c>
+      <c r="J32" s="71">
+        <f>I32+J25+J59</f>
+        <v>4500.4674572184686</v>
+      </c>
+      <c r="K32" s="71">
+        <f>J32+K25+K59</f>
+        <v>5141.1135883943643</v>
+      </c>
+      <c r="L32" s="71">
+        <f>K32+L25+L59</f>
+        <v>5866.4537119655824</v>
+      </c>
+      <c r="M32" s="71">
+        <f>L32+M25+M59</f>
+        <v>6680.7989535967508</v>
       </c>
     </row>
     <row r="33" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -2763,23 +2770,23 @@
       </c>
       <c r="I33" s="40">
         <f>SUM(I31:I32)</f>
-        <v>4219.8903462574999</v>
+        <v>3944.8287250673748</v>
       </c>
       <c r="J33" s="40">
         <f t="shared" ref="J33:M33" si="18">SUM(J31:J32)</f>
-        <v>5099.3345495668746</v>
+        <v>4516.4674572184686</v>
       </c>
       <c r="K33" s="40">
         <f t="shared" si="18"/>
-        <v>6084.9439821451761</v>
+        <v>5157.1135883943643</v>
       </c>
       <c r="L33" s="40">
         <f t="shared" si="18"/>
-        <v>7200.8518645624345</v>
+        <v>5882.4537119655824</v>
       </c>
       <c r="M33" s="40">
         <f t="shared" si="18"/>
-        <v>8453.6906978411553</v>
+        <v>6696.7989535967508</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
@@ -2909,24 +2916,19 @@
         <v>375</v>
       </c>
       <c r="I37" s="20">
-        <f>I7*9.57%</f>
-        <v>412.75649250000009</v>
+        <v>375</v>
       </c>
       <c r="J37" s="20">
-        <f>J7*9.57%</f>
-        <v>454.41832713750011</v>
+        <v>375</v>
       </c>
       <c r="K37" s="20">
-        <f>K7*9.57%</f>
-        <v>500.3361352254376</v>
+        <v>375</v>
       </c>
       <c r="L37" s="20">
-        <f>L7*9.57%</f>
-        <v>548.44773164676019</v>
+        <v>375</v>
       </c>
       <c r="M37" s="20">
-        <f>M7*9.57%</f>
-        <v>599.30624391304116</v>
+        <v>375</v>
       </c>
     </row>
     <row r="38" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -2938,44 +2940,44 @@
         <v>1813</v>
       </c>
       <c r="D38" s="40">
-        <f>SUM(D33:D37)</f>
+        <f t="shared" ref="D38:M38" si="19">SUM(D33:D37)</f>
         <v>2230</v>
       </c>
       <c r="E38" s="40">
-        <f>SUM(E33:E37)</f>
+        <f t="shared" si="19"/>
         <v>2601</v>
       </c>
       <c r="F38" s="40">
-        <f>SUM(F33:F37)</f>
+        <f t="shared" si="19"/>
         <v>3547</v>
       </c>
       <c r="G38" s="40">
-        <f>SUM(G33:G37)</f>
+        <f t="shared" si="19"/>
         <v>3989</v>
       </c>
       <c r="H38" s="40">
-        <f>SUM(H33:H37)</f>
+        <f t="shared" si="19"/>
         <v>4266</v>
       </c>
       <c r="I38" s="40">
-        <f>I33+I36+I37</f>
-        <v>5064.4219990314723</v>
+        <f>SUM(I33:I37)</f>
+        <v>4751.6038853413474</v>
       </c>
       <c r="J38" s="40">
-        <f>J33+J36+J37</f>
-        <v>6029.109532738622</v>
+        <f>SUM(J33:J37)</f>
+        <v>5366.8241132527155</v>
       </c>
       <c r="K38" s="40">
-        <f>K33+K36+K37</f>
-        <v>7108.6703459999635</v>
+        <f>SUM(K33:K37)</f>
+        <v>6055.503817023714</v>
       </c>
       <c r="L38" s="40">
-        <f>L33+L36+L37</f>
-        <v>8290.9879986601536</v>
+        <f>SUM(L33:L37)</f>
+        <v>6799.1421144165415</v>
       </c>
       <c r="M38" s="40">
-        <f>M33+M36+M37</f>
-        <v>9644.9170521161977</v>
+        <f>SUM(M33:M37)</f>
+        <v>7663.7190639587534</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
@@ -3202,27 +3204,28 @@
         <v>388</v>
       </c>
       <c r="H45" s="49">
-        <v>1110</v>
-      </c>
-      <c r="I45" s="20">
+        <f>H63</f>
+        <v>759</v>
+      </c>
+      <c r="I45" s="71">
         <f>I63</f>
-        <v>1502.3307134492243</v>
-      </c>
-      <c r="J45" s="20">
+        <v>1151.3307134492243</v>
+      </c>
+      <c r="J45" s="71">
         <f>J63</f>
-        <v>1944.8814707505749</v>
-      </c>
-      <c r="K45" s="20">
+        <v>1593.8814707505749</v>
+      </c>
+      <c r="K45" s="71">
         <f>K63</f>
-        <v>2431.9989444778325</v>
-      </c>
-      <c r="L45" s="20">
+        <v>2080.9989444778325</v>
+      </c>
+      <c r="L45" s="71">
         <f>L63</f>
-        <v>3033.9617332070748</v>
-      </c>
-      <c r="M45" s="20">
+        <v>2682.9617332070748</v>
+      </c>
+      <c r="M45" s="71">
         <f>M63</f>
-        <v>3686.274173138429</v>
+        <v>3335.274173138429</v>
       </c>
     </row>
     <row r="46" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -3234,43 +3237,44 @@
         <v>1813</v>
       </c>
       <c r="D46" s="40">
-        <f>SUM(D41:D45)</f>
+        <f t="shared" ref="D46:M46" si="20">SUM(D41:D45)</f>
         <v>2230</v>
       </c>
       <c r="E46" s="40">
-        <f>SUM(E41:E45)</f>
+        <f t="shared" si="20"/>
         <v>2601</v>
       </c>
       <c r="F46" s="40">
-        <f>SUM(F41:F45)</f>
+        <f t="shared" si="20"/>
         <v>3547</v>
       </c>
       <c r="G46" s="40">
-        <f>SUM(G41:G45)</f>
+        <f t="shared" si="20"/>
         <v>3989</v>
       </c>
       <c r="H46" s="50">
+        <f>SUM(H41:H45)</f>
         <v>4266</v>
       </c>
       <c r="I46" s="40">
         <f>SUM(I41:I45)</f>
-        <v>5102.6038853413484</v>
+        <v>4751.6038853413484</v>
       </c>
       <c r="J46" s="40">
         <f>SUM(J41:J45)</f>
-        <v>5717.8241132527164</v>
+        <v>5366.8241132527164</v>
       </c>
       <c r="K46" s="40">
         <f>SUM(K41:K45)</f>
-        <v>6406.5038170237149</v>
+        <v>6055.5038170237149</v>
       </c>
       <c r="L46" s="40">
         <f>SUM(L41:L45)</f>
-        <v>7150.1421144165424</v>
+        <v>6799.1421144165424</v>
       </c>
       <c r="M46" s="40">
         <f>SUM(M41:M45)</f>
-        <v>8014.7190639587534</v>
+        <v>7663.7190639587534</v>
       </c>
     </row>
     <row r="47" spans="1:13" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
@@ -3387,19 +3391,19 @@
         <v>785.89034625749991</v>
       </c>
       <c r="J51" s="44">
-        <f t="shared" ref="J51:M51" si="19">J25</f>
+        <f t="shared" ref="J51:M51" si="21">J25</f>
         <v>879.4442033093751</v>
       </c>
       <c r="K51" s="44">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>985.60943257830149</v>
       </c>
       <c r="L51" s="44">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>1115.9078824172586</v>
       </c>
       <c r="M51" s="44">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>1252.8388332787213</v>
       </c>
     </row>
@@ -3431,19 +3435,19 @@
         <v>137.73213187500002</v>
       </c>
       <c r="J52" s="20">
-        <f t="shared" ref="J52:M52" si="20">J18</f>
+        <f t="shared" ref="J52:M52" si="22">J18</f>
         <v>139.58206884375002</v>
       </c>
       <c r="K52" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>142.4033274476719</v>
       </c>
       <c r="L52" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>145.06739624011726</v>
       </c>
       <c r="M52" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>147.84958471784745</v>
       </c>
     </row>
@@ -3519,19 +3523,19 @@
         <v>846.34820963934908</v>
       </c>
       <c r="J54" s="40">
-        <f t="shared" ref="J54:M54" si="21">SUM(J51:J53)</f>
+        <f t="shared" ref="J54:M54" si="23">SUM(J51:J53)</f>
         <v>916.54892908463194</v>
       </c>
       <c r="K54" s="40">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>1015.0668224952883</v>
       </c>
       <c r="L54" s="40">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>1175.9195487528827</v>
       </c>
       <c r="M54" s="40">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>1278.6763274764116</v>
       </c>
     </row>
@@ -3646,19 +3650,19 @@
         <v>-150.95587500000002</v>
       </c>
       <c r="J57" s="40">
-        <f t="shared" ref="J57:M57" si="22">SUM(J55:J56)</f>
+        <f t="shared" ref="J57:M57" si="24">SUM(J55:J56)</f>
         <v>-166.19270062500004</v>
       </c>
       <c r="K57" s="40">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-182.98604736562504</v>
       </c>
       <c r="L57" s="40">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-183.38900117760002</v>
       </c>
       <c r="M57" s="40">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-187.87029589750503</v>
       </c>
     </row>
@@ -3683,7 +3687,7 @@
         <v>-194</v>
       </c>
       <c r="H58" s="40">
-        <v>-350</v>
+        <v>-50</v>
       </c>
       <c r="I58" s="40">
         <v>-28</v>
@@ -3729,19 +3733,19 @@
         <v>-275.06162119012492</v>
       </c>
       <c r="J59" s="20">
-        <f t="shared" ref="J59:M59" si="23">-J51*35%</f>
+        <f t="shared" ref="J59:M59" si="25">-J51*35%</f>
         <v>-307.80547115828125</v>
       </c>
       <c r="K59" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>-344.96330140240548</v>
       </c>
       <c r="L59" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>-390.56775884604048</v>
       </c>
       <c r="M59" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>-438.49359164755242</v>
       </c>
     </row>
@@ -3773,19 +3777,19 @@
         <v>-303.06162119012492</v>
       </c>
       <c r="J60" s="40">
-        <f t="shared" ref="J60:M60" si="24">SUM(J58:J59)</f>
+        <f t="shared" ref="J60:M60" si="26">SUM(J58:J59)</f>
         <v>-307.80547115828125</v>
       </c>
       <c r="K60" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>-344.96330140240548</v>
       </c>
       <c r="L60" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>-390.56775884604048</v>
       </c>
       <c r="M60" s="40">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>-438.49359164755242</v>
       </c>
     </row>
@@ -3810,26 +3814,26 @@
         <v>12</v>
       </c>
       <c r="H61" s="40">
-        <v>173</v>
+        <v>371</v>
       </c>
       <c r="I61" s="40">
         <f>I54+I57+I60</f>
         <v>392.33071344922416</v>
       </c>
       <c r="J61" s="40">
-        <f t="shared" ref="J61:M61" si="25">J54+J57+J60</f>
+        <f t="shared" ref="J61:M61" si="27">J54+J57+J60</f>
         <v>442.55075730135064</v>
       </c>
       <c r="K61" s="40">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>487.11747372725779</v>
       </c>
       <c r="L61" s="40">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>601.96278872924222</v>
       </c>
       <c r="M61" s="40">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>652.31243993135422</v>
       </c>
     </row>
@@ -3854,27 +3858,28 @@
         <v>234</v>
       </c>
       <c r="H62" s="40">
-        <v>937</v>
+        <f>G45</f>
+        <v>388</v>
       </c>
       <c r="I62" s="40">
         <f>H63</f>
-        <v>1110</v>
+        <v>759</v>
       </c>
       <c r="J62" s="40">
         <f>I63</f>
-        <v>1502.3307134492243</v>
+        <v>1151.3307134492243</v>
       </c>
       <c r="K62" s="40">
         <f>J63</f>
-        <v>1944.8814707505749</v>
+        <v>1593.8814707505749</v>
       </c>
       <c r="L62" s="40">
         <f>K63</f>
-        <v>2431.9989444778325</v>
+        <v>2080.9989444778325</v>
       </c>
       <c r="M62" s="40">
         <f>L63</f>
-        <v>3033.9617332070748</v>
+        <v>2682.9617332070748</v>
       </c>
     </row>
     <row r="63" spans="1:13" s="43" customFormat="1" x14ac:dyDescent="0.3">
@@ -3898,27 +3903,28 @@
         <v>388</v>
       </c>
       <c r="H63" s="40">
-        <v>1110</v>
+        <f>H61+H62</f>
+        <v>759</v>
       </c>
       <c r="I63" s="40">
-        <f>I61+I62</f>
-        <v>1502.3307134492243</v>
+        <f t="shared" ref="H63:M63" si="28">I61+I62</f>
+        <v>1151.3307134492243</v>
       </c>
       <c r="J63" s="40">
-        <f>J61+J62</f>
-        <v>1944.8814707505749</v>
+        <f t="shared" si="28"/>
+        <v>1593.8814707505749</v>
       </c>
       <c r="K63" s="40">
-        <f>K61+K62</f>
-        <v>2431.9989444778325</v>
+        <f t="shared" si="28"/>
+        <v>2080.9989444778325</v>
       </c>
       <c r="L63" s="40">
-        <f>L61+L62</f>
-        <v>3033.9617332070748</v>
+        <f t="shared" si="28"/>
+        <v>2682.9617332070748</v>
       </c>
       <c r="M63" s="40">
-        <f>M61+M62</f>
-        <v>3686.274173138429</v>
+        <f t="shared" si="28"/>
+        <v>3335.274173138429</v>
       </c>
     </row>
   </sheetData>
@@ -3953,13 +3959,13 @@
       <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
@@ -4191,11 +4197,11 @@
       <c r="H12" s="14"/>
     </row>
     <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="76" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="74"/>
-      <c r="C13" s="74"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="76"/>
       <c r="D13" s="26"/>
       <c r="E13" s="26"/>
       <c r="F13" s="15"/>
@@ -4337,11 +4343,11 @@
       <c r="H20" s="14"/>
     </row>
     <row r="21" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A21" s="70" t="s">
+      <c r="A21" s="72" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="70"/>
-      <c r="C21" s="70"/>
+      <c r="B21" s="72"/>
+      <c r="C21" s="72"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
       <c r="F21" s="15"/>
@@ -4608,13 +4614,13 @@
       <c r="H32" s="14"/>
     </row>
     <row r="33" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A33" s="70" t="s">
+      <c r="A33" s="72" t="s">
         <v>61</v>
       </c>
-      <c r="B33" s="70"/>
-      <c r="C33" s="70"/>
-      <c r="D33" s="70"/>
-      <c r="E33" s="70"/>
+      <c r="B33" s="72"/>
+      <c r="C33" s="72"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="72"/>
       <c r="F33" s="15"/>
       <c r="G33" s="15"/>
       <c r="H33" s="15"/>
@@ -4801,11 +4807,11 @@
       <c r="H41" s="14"/>
     </row>
     <row r="42" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A42" s="70" t="s">
+      <c r="A42" s="72" t="s">
         <v>67</v>
       </c>
-      <c r="B42" s="70"/>
-      <c r="C42" s="70"/>
+      <c r="B42" s="72"/>
+      <c r="C42" s="72"/>
       <c r="D42" s="32"/>
       <c r="E42" s="15"/>
       <c r="F42" s="15"/>
@@ -5006,11 +5012,11 @@
       <c r="K1" s="22"/>
     </row>
     <row r="2" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
       <c r="D2" s="15"/>
       <c r="E2" s="15"/>
       <c r="F2" s="15"/>
@@ -5021,9 +5027,9 @@
       <c r="K2" s="14"/>
     </row>
     <row r="3" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="70"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
+      <c r="A3" s="72"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
@@ -5271,11 +5277,11 @@
       <c r="K12" s="14"/>
     </row>
     <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="70" t="s">
+      <c r="A13" s="72" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="70"/>
-      <c r="C13" s="70"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
@@ -5286,9 +5292,9 @@
       <c r="K13" s="14"/>
     </row>
     <row r="14" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="70"/>
-      <c r="B14" s="70"/>
-      <c r="C14" s="70"/>
+      <c r="A14" s="72"/>
+      <c r="B14" s="72"/>
+      <c r="C14" s="72"/>
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
@@ -5502,11 +5508,11 @@
       <c r="K26" s="14"/>
     </row>
     <row r="27" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="70" t="s">
+      <c r="A27" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="B27" s="70"/>
-      <c r="C27" s="70"/>
+      <c r="B27" s="72"/>
+      <c r="C27" s="72"/>
       <c r="D27" s="15"/>
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
@@ -5517,9 +5523,9 @@
       <c r="K27" s="14"/>
     </row>
     <row r="28" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="70"/>
-      <c r="B28" s="70"/>
-      <c r="C28" s="70"/>
+      <c r="A28" s="72"/>
+      <c r="B28" s="72"/>
+      <c r="C28" s="72"/>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
@@ -5833,14 +5839,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="72" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="34"/>
       <c r="H1" s="34"/>
       <c r="I1" s="34"/>
@@ -5848,12 +5854,12 @@
       <c r="K1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="75"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
       <c r="G2" s="34"/>
       <c r="H2" s="34"/>
       <c r="I2" s="34"/>

</xml_diff>